<commit_message>
chore: sync user edited customers.xlsx and clean sample files
</commit_message>
<xml_diff>
--- a/apps/web/public/samples/customers.xlsx
+++ b/apps/web/public/samples/customers.xlsx
@@ -1,12 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
+  <bookViews>
+    <workbookView windowWidth="19200" windowHeight="6200"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Customers" state="visible" r:id="rId4"/>
+    <sheet name="Customers" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -43,7 +59,7 @@
     <t>Example Cafe Ltd</t>
   </si>
   <si>
-    <t>orders@example-cafe.example</t>
+    <t>amirmaqbool055@gmail.com</t>
   </si>
   <si>
     <t>example-cafe.example</t>
@@ -67,7 +83,7 @@
     <t>Apex Fine Dining Group</t>
   </si>
   <si>
-    <t>procurement@apexdining.co.uk</t>
+    <t>amirmaqbortol055@gmail.com</t>
   </si>
   <si>
     <t>apexdining.co.uk</t>
@@ -88,7 +104,7 @@
     <t>The Highland Bistro</t>
   </si>
   <si>
-    <t>orders@highlandbistro.co.uk</t>
+    <t>amirvsvxcmaqbool055@gmail.com</t>
   </si>
   <si>
     <t>highlandbistro.co.uk</t>
@@ -109,7 +125,7 @@
     <t>Bayside Fish &amp; Grill</t>
   </si>
   <si>
-    <t>supplies@baysidegrill.com</t>
+    <t>amirmadfdfdvqbool055@gmail.com</t>
   </si>
   <si>
     <t>baysidegrill.com</t>
@@ -130,7 +146,7 @@
     <t>Riverside Artisan Bakery</t>
   </si>
   <si>
-    <t>bake@riversidebakery.co.uk</t>
+    <t>amirmaqbovvxcvxcol055@gmail.com</t>
   </si>
   <si>
     <t>riversidebakery.co.uk</t>
@@ -169,21 +185,182 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
-    <font>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="42" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="22">
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -193,10 +370,197 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1E293B"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -204,27 +568,315 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -546,14 +1198,14 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="6" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -564,7 +1216,7 @@
     <col min="7" max="8" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" s="1" customFormat="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -590,14 +1242,14 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
         <v>8</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D2" t="s">
@@ -616,14 +1268,14 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
         <v>16</v>
       </c>
       <c r="B3" t="s">
         <v>17</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D3" t="s">
@@ -642,14 +1294,14 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
         <v>23</v>
       </c>
       <c r="B4" t="s">
         <v>24</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D4" t="s">
@@ -668,14 +1320,14 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
         <v>30</v>
       </c>
       <c r="B5" t="s">
         <v>31</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="3" t="s">
         <v>32</v>
       </c>
       <c r="D5" t="s">
@@ -694,14 +1346,14 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
         <v>37</v>
       </c>
       <c r="B6" t="s">
         <v>38</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="3" t="s">
         <v>39</v>
       </c>
       <c r="D6" t="s">
@@ -720,14 +1372,14 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
         <v>44</v>
       </c>
       <c r="B7" t="s">
         <v>45</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="2" t="s">
         <v>46</v>
       </c>
       <c r="D7" t="s">
@@ -747,7 +1399,16 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" display="amirmaqbool055@gmail.com"/>
+    <hyperlink ref="C3" r:id="rId2" display="amirmaqbortol055@gmail.com" tooltip="mailto:amirmaqbortol055@gmail.com"/>
+    <hyperlink ref="C4" r:id="rId3" display="amirvsvxcmaqbool055@gmail.com" tooltip="mailto:amirvsvxcmaqbool055@gmail.com"/>
+    <hyperlink ref="C5" r:id="rId4" display="amirmadfdfdvqbool055@gmail.com" tooltip="mailto:amirmadfdfdvqbool055@gmail.com"/>
+    <hyperlink ref="C6" r:id="rId5" display="amirmaqbovvxcvxcol055@gmail.com" tooltip="mailto:amirmaqbovvxcvxcol055@gmail.com"/>
+    <hyperlink ref="C7" r:id="rId6" display="purchasing@metrohotel.com"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>